<commit_message>
Update data/schools.xlsx from EditExcel
</commit_message>
<xml_diff>
--- a/data/schools.xlsx
+++ b/data/schools.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Walid\Downloads\بيانات المدارس\بيانات المدارس\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Walid\AppData\Local\EditExcel\Sessions\BB0303897D6B9842BF4B3EAA\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="210">
   <si>
     <t>اسم المدرسة</t>
   </si>
@@ -646,6 +646,9 @@
   </si>
   <si>
     <t>https://maps.app.goo.gl/Fgmcb6q96A6XPxEh6</t>
+  </si>
+  <si>
+    <t>محمد علي كلاي</t>
   </si>
 </sst>
 </file>
@@ -1868,7 +1871,9 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="27.95" customHeight="1">
-      <c r="A28" s="1"/>
+      <c r="A28" s="1" t="s">
+        <v>209</v>
+      </c>
       <c r="B28" s="1"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>

</xml_diff>